<commit_message>
updated light exposure trial dates and removed duplicates
</commit_message>
<xml_diff>
--- a/data/Study_dates_MeLiDos_KNUST.xlsx
+++ b/data/Study_dates_MeLiDos_KNUST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\MeLiDos\MeLiDos_KNUST\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zauner/Documents/Arbeit/12-TUM/MeLiDos/WP2.2.5_Data_Analysis/AkuffoEtAl_Dataset_2025/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93A014D9-4035-4019-80AC-074111FCA09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FAA18E-7A8C-874A-83E9-85B0925BCDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{6C9F1A2F-5B37-46DB-8DE9-38CAE235C339}"/>
+    <workbookView xWindow="59620" yWindow="3440" windowWidth="31800" windowHeight="19340" xr2:uid="{6C9F1A2F-5B37-46DB-8DE9-38CAE235C339}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -201,6 +201,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -231,14 +232,14 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{4B83247E-72C7-487E-B57F-2C325B5C7841}"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -254,9 +255,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -294,7 +295,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -400,7 +401,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -542,7 +543,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -551,16 +552,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C398934C-0708-4D30-BA98-2C46610FD8D7}">
   <dimension ref="A1:E60"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -577,7 +578,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -588,13 +589,13 @@
         <v>10</v>
       </c>
       <c r="D2" s="4">
-        <v>45573.375</v>
+        <v>45572.5</v>
       </c>
       <c r="E2" s="4">
-        <v>45579.390972222223</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45579.458333333336</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -605,13 +606,13 @@
         <v>10</v>
       </c>
       <c r="D3" s="4">
-        <v>45573.375</v>
+        <v>45572.5</v>
       </c>
       <c r="E3" s="4">
-        <v>45579.390972222223</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45579.458333333336</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -622,18 +623,18 @@
         <v>10</v>
       </c>
       <c r="D4" s="4">
-        <v>45573.375</v>
+        <v>45572.5</v>
       </c>
       <c r="E4" s="4">
-        <v>45579.390972222223</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45579.458333333336</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
     </row>
-    <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -644,13 +645,13 @@
         <v>10</v>
       </c>
       <c r="D6" s="4">
-        <v>45580.29583333333</v>
+        <v>45579.79583333333</v>
       </c>
       <c r="E6" s="4">
-        <v>45585.936805555553</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45586.416666666664</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -661,13 +662,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="4">
-        <v>45580.29583333333</v>
+        <v>45579.79583333333</v>
       </c>
       <c r="E7" s="4">
-        <v>45585.936805555553</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45586.416666666664</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -678,18 +679,18 @@
         <v>10</v>
       </c>
       <c r="D8" s="4">
-        <v>45580.29583333333</v>
+        <v>45579.79583333333</v>
       </c>
       <c r="E8" s="4">
-        <v>45585.936805555553</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45586.416666666664</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
     </row>
-    <row r="10" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
@@ -700,13 +701,13 @@
         <v>10</v>
       </c>
       <c r="D10" s="4">
-        <v>45587.289583333331</v>
+        <v>45586.622916666667</v>
       </c>
       <c r="E10" s="4">
-        <v>45592.838888888888</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45593.416666666664</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
@@ -717,13 +718,13 @@
         <v>10</v>
       </c>
       <c r="D11" s="4">
-        <v>45587.289583333331</v>
+        <v>45586.622916666667</v>
       </c>
       <c r="E11" s="4">
-        <v>45592.838888888888</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45593.416666666664</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
@@ -734,18 +735,18 @@
         <v>10</v>
       </c>
       <c r="D12" s="4">
-        <v>45587.289583333331</v>
+        <v>45586.622916666667</v>
       </c>
       <c r="E12" s="4">
-        <v>45592.838888888888</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45593.416666666664</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
@@ -756,13 +757,13 @@
         <v>10</v>
       </c>
       <c r="D14" s="4">
-        <v>45594.256944444445</v>
+        <v>45593.756944444445</v>
       </c>
       <c r="E14" s="4">
-        <v>45599.329861111109</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45600.458333333336</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
@@ -773,13 +774,13 @@
         <v>10</v>
       </c>
       <c r="D15" s="4">
-        <v>45594.256944444445</v>
+        <v>45593.756944444445</v>
       </c>
       <c r="E15" s="4">
-        <v>45599.329861111109</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45600.458333333336</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>16</v>
       </c>
@@ -790,18 +791,18 @@
         <v>10</v>
       </c>
       <c r="D16" s="4">
-        <v>45594.256944444445</v>
+        <v>45593.756944444445</v>
       </c>
       <c r="E16" s="4">
-        <v>45599.329861111109</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45600.458333333336</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
     </row>
-    <row r="18" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>17</v>
       </c>
@@ -812,13 +813,13 @@
         <v>10</v>
       </c>
       <c r="D18" s="4">
-        <v>45601.290972222225</v>
+        <v>45600.5</v>
       </c>
       <c r="E18" s="4">
         <v>45607.368055555555</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>18</v>
       </c>
@@ -829,13 +830,13 @@
         <v>10</v>
       </c>
       <c r="D19" s="4">
-        <v>45601.290972222225</v>
+        <v>45600.5</v>
       </c>
       <c r="E19" s="4">
         <v>45607.368055555555</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>19</v>
       </c>
@@ -846,18 +847,18 @@
         <v>10</v>
       </c>
       <c r="D20" s="4">
-        <v>45601.290972222225</v>
+        <v>45600.5</v>
       </c>
       <c r="E20" s="4">
         <v>45607.368055555555</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
     </row>
-    <row r="22" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
@@ -868,13 +869,13 @@
         <v>10</v>
       </c>
       <c r="D22" s="4">
-        <v>45608.277777777781</v>
+        <v>45607.583333333336</v>
       </c>
       <c r="E22" s="4">
-        <v>45614.377083333333</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45614.418749999997</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
@@ -885,13 +886,13 @@
         <v>10</v>
       </c>
       <c r="D23" s="4">
-        <v>45608.277777777781</v>
+        <v>45607.583333333336</v>
       </c>
       <c r="E23" s="4">
-        <v>45614.377083333333</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45614.418749999997</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
@@ -902,18 +903,18 @@
         <v>10</v>
       </c>
       <c r="D24" s="4">
-        <v>45608.277777777781</v>
+        <v>45607.583333333336</v>
       </c>
       <c r="E24" s="4">
-        <v>45614.377083333333</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45614.418749999997</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
     </row>
-    <row r="26" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>22</v>
       </c>
@@ -924,13 +925,13 @@
         <v>10</v>
       </c>
       <c r="D26" s="4">
-        <v>45615.330555555556</v>
+        <v>45614.625</v>
       </c>
       <c r="E26" s="4">
         <v>45621.422222222223</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>23</v>
       </c>
@@ -941,13 +942,13 @@
         <v>10</v>
       </c>
       <c r="D27" s="4">
-        <v>45615.330555555556</v>
+        <v>45614.625</v>
       </c>
       <c r="E27" s="4">
         <v>45621.422222222223</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>24</v>
       </c>
@@ -958,18 +959,18 @@
         <v>10</v>
       </c>
       <c r="D28" s="4">
-        <v>45615.330555555556</v>
+        <v>45614.625</v>
       </c>
       <c r="E28" s="4">
         <v>45621.422222222223</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
     </row>
-    <row r="30" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
@@ -980,13 +981,13 @@
         <v>10</v>
       </c>
       <c r="D30" s="4">
-        <v>45622.319444444445</v>
+        <v>45621.583333333336</v>
       </c>
       <c r="E30" s="4">
-        <v>45628.375694444447</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45628.459027777775</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>26</v>
       </c>
@@ -997,13 +998,13 @@
         <v>10</v>
       </c>
       <c r="D31" s="4">
-        <v>45622.319444444445</v>
+        <v>45621.583333333336</v>
       </c>
       <c r="E31" s="4">
-        <v>45628.375694444447</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45628.459027777775</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>27</v>
       </c>
@@ -1014,18 +1015,18 @@
         <v>10</v>
       </c>
       <c r="D32" s="4">
-        <v>45622.319444444445</v>
+        <v>45621.583333333336</v>
       </c>
       <c r="E32" s="4">
-        <v>45628.375694444447</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45628.459027777775</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="3"/>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
     </row>
-    <row r="34" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>28</v>
       </c>
@@ -1036,13 +1037,13 @@
         <v>10</v>
       </c>
       <c r="D34" s="4">
-        <v>45629.364583333336</v>
+        <v>45628.53125</v>
       </c>
       <c r="E34" s="4">
-        <v>45635.376388888886</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45635.418055555558</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>29</v>
       </c>
@@ -1053,13 +1054,13 @@
         <v>10</v>
       </c>
       <c r="D35" s="4">
-        <v>45629.364583333336</v>
+        <v>45628.53125</v>
       </c>
       <c r="E35" s="4">
-        <v>45635.376388888886</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45635.418055555558</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>30</v>
       </c>
@@ -1070,18 +1071,18 @@
         <v>10</v>
       </c>
       <c r="D36" s="4">
-        <v>45629.364583333336</v>
+        <v>45628.53125</v>
       </c>
       <c r="E36" s="4">
-        <v>45635.376388888886</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45635.418055555558</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
-    <row r="38" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>48</v>
       </c>
@@ -1092,13 +1093,13 @@
         <v>10</v>
       </c>
       <c r="D38" s="4">
-        <v>45636.338194444441</v>
+        <v>45635.520833333336</v>
       </c>
       <c r="E38" s="4">
-        <v>45642.368055555555</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45642.409722222219</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>47</v>
       </c>
@@ -1109,13 +1110,13 @@
         <v>10</v>
       </c>
       <c r="D39" s="4">
-        <v>45636.338194444441</v>
+        <v>45635.520833333336</v>
       </c>
       <c r="E39" s="4">
-        <v>45642.368055555555</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45642.409722222219</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>46</v>
       </c>
@@ -1126,18 +1127,18 @@
         <v>10</v>
       </c>
       <c r="D40" s="4">
-        <v>45636.338194444441</v>
+        <v>45635.520833333336</v>
       </c>
       <c r="E40" s="4">
-        <v>45642.368055555555</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45642.409722222219</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
-    <row r="42" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>44</v>
       </c>
@@ -1148,13 +1149,13 @@
         <v>10</v>
       </c>
       <c r="D42" s="4">
-        <v>45643.304166666669</v>
+        <v>45642.595833333333</v>
       </c>
       <c r="E42" s="4">
-        <v>45649.348611111112</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45649.390277777777</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>45</v>
       </c>
@@ -1165,13 +1166,13 @@
         <v>10</v>
       </c>
       <c r="D43" s="4">
-        <v>45643.304166666669</v>
+        <v>45642.595833333333</v>
       </c>
       <c r="E43" s="4">
-        <v>45649.348611111112</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45649.390277777777</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>43</v>
       </c>
@@ -1182,18 +1183,18 @@
         <v>10</v>
       </c>
       <c r="D44" s="4">
-        <v>45643.304166666669</v>
+        <v>45642.595833333333</v>
       </c>
       <c r="E44" s="4">
-        <v>45649.348611111112</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45649.390277777777</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="3"/>
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
     </row>
-    <row r="46" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>42</v>
       </c>
@@ -1204,13 +1205,13 @@
         <v>10</v>
       </c>
       <c r="D46" s="4">
-        <v>45664.293055555558</v>
+        <v>45663.584722222222</v>
       </c>
       <c r="E46" s="4">
-        <v>45670.386111111111</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45670.427777777775</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
         <v>41</v>
       </c>
@@ -1221,13 +1222,13 @@
         <v>10</v>
       </c>
       <c r="D47" s="4">
-        <v>45664.293055555558</v>
+        <v>45663.584722222222</v>
       </c>
       <c r="E47" s="4">
-        <v>45670.386111111111</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45670.427777777775</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>40</v>
       </c>
@@ -1238,18 +1239,18 @@
         <v>10</v>
       </c>
       <c r="D48" s="4">
-        <v>45664.293055555558</v>
+        <v>45663.584722222222</v>
       </c>
       <c r="E48" s="4">
-        <v>45670.386111111111</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45670.427777777775</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="3"/>
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
     </row>
-    <row r="50" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>39</v>
       </c>
@@ -1260,13 +1261,13 @@
         <v>10</v>
       </c>
       <c r="D50" s="4">
-        <v>45671.974305555559</v>
+        <v>45670.583333333336</v>
       </c>
       <c r="E50" s="4">
         <v>45677.4375</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>38</v>
       </c>
@@ -1277,13 +1278,13 @@
         <v>10</v>
       </c>
       <c r="D51" s="4">
-        <v>45671.974305555559</v>
+        <v>45670.583333333336</v>
       </c>
       <c r="E51" s="4">
         <v>45677.4375</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>37</v>
       </c>
@@ -1294,18 +1295,18 @@
         <v>10</v>
       </c>
       <c r="D52" s="4">
-        <v>45671.974305555559</v>
+        <v>45670.583333333336</v>
       </c>
       <c r="E52" s="4">
         <v>45677.4375</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="3"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
     </row>
-    <row r="54" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>36</v>
       </c>
@@ -1316,13 +1317,13 @@
         <v>10</v>
       </c>
       <c r="D54" s="4">
-        <v>45679.313194444447</v>
+        <v>45677.313194444447</v>
       </c>
       <c r="E54" s="4">
         <v>45684.463194444441</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
         <v>35</v>
       </c>
@@ -1333,13 +1334,13 @@
         <v>10</v>
       </c>
       <c r="D55" s="4">
-        <v>45679.313194444447</v>
+        <v>45677.313194444447</v>
       </c>
       <c r="E55" s="4">
         <v>45684.463194444441</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>34</v>
       </c>
@@ -1350,18 +1351,18 @@
         <v>10</v>
       </c>
       <c r="D56" s="4">
-        <v>45679.313194444447</v>
+        <v>45677.313194444447</v>
       </c>
       <c r="E56" s="4">
         <v>45684.463194444441</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="3"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
     </row>
-    <row r="58" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>33</v>
       </c>
@@ -1372,13 +1373,13 @@
         <v>10</v>
       </c>
       <c r="D58" s="4">
-        <v>45685.291666666664</v>
+        <v>45684.291666666664</v>
       </c>
       <c r="E58" s="4">
-        <v>45691.503472222219</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45718.503472222219</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
         <v>32</v>
       </c>
@@ -1389,13 +1390,13 @@
         <v>10</v>
       </c>
       <c r="D59" s="4">
-        <v>45685.291666666664</v>
+        <v>45684.291666666664</v>
       </c>
       <c r="E59" s="4">
-        <v>45691.503472222219</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>45718.503472222219</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>31</v>
       </c>
@@ -1406,10 +1407,10 @@
         <v>10</v>
       </c>
       <c r="D60" s="4">
-        <v>45685.291666666664</v>
+        <v>45684.291666666664</v>
       </c>
       <c r="E60" s="4">
-        <v>45691.503472222219</v>
+        <v>45718.503472222219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>